<commit_message>
Atualização de alguma coisa
</commit_message>
<xml_diff>
--- a/exibir_NF/invoice-processor/spreadsheets/Card_Alinemptosta_7221_MAIO_2026.xlsx
+++ b/exibir_NF/invoice-processor/spreadsheets/Card_Alinemptosta_7221_MAIO_2026.xlsx
@@ -710,11 +710,25 @@
       <c r="K5" s="22" t="n"/>
     </row>
     <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="20" t="n"/>
+      <c r="A6" s="20" t="inlineStr">
+        <is>
+          <t>16/04</t>
+        </is>
+      </c>
       <c r="B6" s="21" t="n"/>
-      <c r="C6" s="22" t="n"/>
-      <c r="D6" s="22" t="n"/>
-      <c r="E6" s="23" t="n"/>
+      <c r="C6" s="22" t="inlineStr">
+        <is>
+          <t>PANIFESTRDOBUTANTA</t>
+        </is>
+      </c>
+      <c r="D6" s="22" t="inlineStr">
+        <is>
+          <t>PANIFESTRDOBUTANTA</t>
+        </is>
+      </c>
+      <c r="E6" s="23" t="n">
+        <v>130.51</v>
+      </c>
       <c r="F6" s="21" t="inlineStr">
         <is>
           <t>A VISTA</t>
@@ -727,11 +741,25 @@
       <c r="K6" s="22" t="n"/>
     </row>
     <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="20" t="n"/>
+      <c r="A7" s="20" t="inlineStr">
+        <is>
+          <t>17/04</t>
+        </is>
+      </c>
       <c r="B7" s="21" t="n"/>
-      <c r="C7" s="22" t="n"/>
-      <c r="D7" s="22" t="n"/>
-      <c r="E7" s="23" t="n"/>
+      <c r="C7" s="22" t="inlineStr">
+        <is>
+          <t>DL*UberRides</t>
+        </is>
+      </c>
+      <c r="D7" s="22" t="inlineStr">
+        <is>
+          <t>DL*UberRides</t>
+        </is>
+      </c>
+      <c r="E7" s="23" t="n">
+        <v>37.58</v>
+      </c>
       <c r="F7" s="21" t="inlineStr">
         <is>
           <t>A VISTA</t>
@@ -744,11 +772,25 @@
       <c r="K7" s="22" t="n"/>
     </row>
     <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="20" t="n"/>
+      <c r="A8" s="20" t="inlineStr">
+        <is>
+          <t>17/04</t>
+        </is>
+      </c>
       <c r="B8" s="21" t="n"/>
-      <c r="C8" s="22" t="n"/>
-      <c r="D8" s="22" t="n"/>
-      <c r="E8" s="23" t="n"/>
+      <c r="C8" s="22" t="inlineStr">
+        <is>
+          <t>MERCADOLIVRE*NILSON</t>
+        </is>
+      </c>
+      <c r="D8" s="22" t="inlineStr">
+        <is>
+          <t>MERCADOLIVRE*NILSON</t>
+        </is>
+      </c>
+      <c r="E8" s="23" t="n">
+        <v>468.42</v>
+      </c>
       <c r="F8" s="21" t="inlineStr">
         <is>
           <t>A VISTA</t>
@@ -761,11 +803,25 @@
       <c r="K8" s="22" t="n"/>
     </row>
     <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="20" t="n"/>
+      <c r="A9" s="20" t="inlineStr">
+        <is>
+          <t>17/04</t>
+        </is>
+      </c>
       <c r="B9" s="21" t="n"/>
-      <c r="C9" s="22" t="n"/>
-      <c r="D9" s="22" t="n"/>
-      <c r="E9" s="23" t="n"/>
+      <c r="C9" s="22" t="inlineStr">
+        <is>
+          <t>PANIFESTRDOBUTANTA</t>
+        </is>
+      </c>
+      <c r="D9" s="22" t="inlineStr">
+        <is>
+          <t>PANIFESTRDOBUTANTA</t>
+        </is>
+      </c>
+      <c r="E9" s="23" t="n">
+        <v>140.37</v>
+      </c>
       <c r="F9" s="21" t="inlineStr">
         <is>
           <t>A VISTA</t>
@@ -778,11 +834,25 @@
       <c r="K9" s="22" t="n"/>
     </row>
     <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="20" t="n"/>
+      <c r="A10" s="20" t="inlineStr">
+        <is>
+          <t>18/04</t>
+        </is>
+      </c>
       <c r="B10" s="21" t="n"/>
-      <c r="C10" s="22" t="n"/>
-      <c r="D10" s="22" t="n"/>
-      <c r="E10" s="23" t="n"/>
+      <c r="C10" s="22" t="inlineStr">
+        <is>
+          <t>STARLINKINTERNET</t>
+        </is>
+      </c>
+      <c r="D10" s="22" t="inlineStr">
+        <is>
+          <t>STARLINKINTERNET</t>
+        </is>
+      </c>
+      <c r="E10" s="23" t="n">
+        <v>576</v>
+      </c>
       <c r="F10" s="21" t="inlineStr">
         <is>
           <t>A VISTA</t>
@@ -795,11 +865,25 @@
       <c r="K10" s="22" t="n"/>
     </row>
     <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="20" t="n"/>
+      <c r="A11" s="20" t="inlineStr">
+        <is>
+          <t>20/04</t>
+        </is>
+      </c>
       <c r="B11" s="21" t="n"/>
-      <c r="C11" s="22" t="n"/>
-      <c r="D11" s="22" t="n"/>
-      <c r="E11" s="23" t="n"/>
+      <c r="C11" s="22" t="inlineStr">
+        <is>
+          <t>STARLINKINTERNET</t>
+        </is>
+      </c>
+      <c r="D11" s="22" t="inlineStr">
+        <is>
+          <t>STARLINKINTERNET</t>
+        </is>
+      </c>
+      <c r="E11" s="23" t="n">
+        <v>576</v>
+      </c>
       <c r="F11" s="21" t="inlineStr">
         <is>
           <t>A VISTA</t>
@@ -812,11 +896,25 @@
       <c r="K11" s="22" t="n"/>
     </row>
     <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="20" t="n"/>
+      <c r="A12" s="20" t="inlineStr">
+        <is>
+          <t>20/04</t>
+        </is>
+      </c>
       <c r="B12" s="21" t="n"/>
-      <c r="C12" s="22" t="n"/>
-      <c r="D12" s="22" t="n"/>
-      <c r="E12" s="23" t="n"/>
+      <c r="C12" s="22" t="inlineStr">
+        <is>
+          <t>STARLINKINTERNET</t>
+        </is>
+      </c>
+      <c r="D12" s="22" t="inlineStr">
+        <is>
+          <t>STARLINKINTERNET</t>
+        </is>
+      </c>
+      <c r="E12" s="23" t="n">
+        <v>576</v>
+      </c>
       <c r="F12" s="21" t="inlineStr">
         <is>
           <t>A VISTA</t>
@@ -829,11 +927,25 @@
       <c r="K12" s="22" t="n"/>
     </row>
     <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="20" t="n"/>
+      <c r="A13" s="20" t="inlineStr">
+        <is>
+          <t>22/04</t>
+        </is>
+      </c>
       <c r="B13" s="21" t="n"/>
-      <c r="C13" s="22" t="n"/>
-      <c r="D13" s="22" t="n"/>
-      <c r="E13" s="23" t="n"/>
+      <c r="C13" s="22" t="inlineStr">
+        <is>
+          <t>PPRO *MICROSOFT</t>
+        </is>
+      </c>
+      <c r="D13" s="22" t="inlineStr">
+        <is>
+          <t>PPRO *MICROSOFT</t>
+        </is>
+      </c>
+      <c r="E13" s="23" t="n">
+        <v>60</v>
+      </c>
       <c r="F13" s="21" t="inlineStr">
         <is>
           <t>A VISTA</t>
@@ -846,11 +958,25 @@
       <c r="K13" s="22" t="n"/>
     </row>
     <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="20" t="n"/>
+      <c r="A14" s="20" t="inlineStr">
+        <is>
+          <t>22/04</t>
+        </is>
+      </c>
       <c r="B14" s="21" t="n"/>
-      <c r="C14" s="22" t="n"/>
-      <c r="D14" s="22" t="n"/>
-      <c r="E14" s="23" t="n"/>
+      <c r="C14" s="22" t="inlineStr">
+        <is>
+          <t>SUPERMERCADOPADRAO</t>
+        </is>
+      </c>
+      <c r="D14" s="22" t="inlineStr">
+        <is>
+          <t>SUPERMERCADOPADRAO</t>
+        </is>
+      </c>
+      <c r="E14" s="23" t="n">
+        <v>524.42</v>
+      </c>
       <c r="F14" s="21" t="inlineStr">
         <is>
           <t>A VISTA</t>
@@ -863,11 +989,25 @@
       <c r="K14" s="22" t="n"/>
     </row>
     <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="20" t="n"/>
+      <c r="A15" s="20" t="inlineStr">
+        <is>
+          <t>22/04</t>
+        </is>
+      </c>
       <c r="B15" s="21" t="n"/>
-      <c r="C15" s="22" t="n"/>
-      <c r="D15" s="22" t="n"/>
-      <c r="E15" s="23" t="n"/>
+      <c r="C15" s="22" t="inlineStr">
+        <is>
+          <t>DL *UberRides</t>
+        </is>
+      </c>
+      <c r="D15" s="22" t="inlineStr">
+        <is>
+          <t>DL *UberRides</t>
+        </is>
+      </c>
+      <c r="E15" s="23" t="n">
+        <v>20.95</v>
+      </c>
       <c r="F15" s="21" t="inlineStr">
         <is>
           <t>A VISTA</t>
@@ -880,11 +1020,25 @@
       <c r="K15" s="22" t="n"/>
     </row>
     <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="20" t="n"/>
+      <c r="A16" s="20" t="inlineStr">
+        <is>
+          <t>23/04</t>
+        </is>
+      </c>
       <c r="B16" s="21" t="n"/>
-      <c r="C16" s="22" t="n"/>
-      <c r="D16" s="22" t="n"/>
-      <c r="E16" s="23" t="n"/>
+      <c r="C16" s="22" t="inlineStr">
+        <is>
+          <t>MERCADOLIVRE*PRESENTE</t>
+        </is>
+      </c>
+      <c r="D16" s="22" t="inlineStr">
+        <is>
+          <t>MERCADOLIVRE*PRESENTE</t>
+        </is>
+      </c>
+      <c r="E16" s="23" t="n">
+        <v>1579.8</v>
+      </c>
       <c r="F16" s="21" t="inlineStr">
         <is>
           <t>A VISTA</t>
@@ -897,52 +1051,66 @@
       <c r="K16" s="22" t="n"/>
     </row>
     <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="5" t="inlineStr">
+      <c r="A17" s="20" t="inlineStr">
+        <is>
+          <t>23/04</t>
+        </is>
+      </c>
+      <c r="B17" s="21" t="n"/>
+      <c r="C17" s="22" t="inlineStr">
+        <is>
+          <t>MERCADOLIVRE*PROTEC</t>
+        </is>
+      </c>
+      <c r="D17" s="22" t="inlineStr">
+        <is>
+          <t>MERCADOLIVRE*PROTEC</t>
+        </is>
+      </c>
+      <c r="E17" s="23" t="n">
+        <v>123.25</v>
+      </c>
+      <c r="F17" s="21" t="inlineStr">
+        <is>
+          <t>A VISTA</t>
+        </is>
+      </c>
+      <c r="G17" s="21" t="n"/>
+      <c r="H17" s="22" t="n"/>
+      <c r="I17" s="21" t="n"/>
+      <c r="J17" s="22" t="n"/>
+      <c r="K17" s="22" t="n"/>
+    </row>
+    <row r="18" ht="18" customHeight="1">
+      <c r="A18" s="20" t="inlineStr">
         <is>
           <t>24/04</t>
         </is>
       </c>
-      <c r="B17" s="6" t="n"/>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="B18" s="21" t="n"/>
+      <c r="C18" s="22" t="inlineStr">
         <is>
           <t>MERCADOLIVRE*MERCADOL</t>
         </is>
       </c>
-      <c r="D17" s="3" t="inlineStr">
+      <c r="D18" s="22" t="inlineStr">
         <is>
           <t>MERCADOLIVRE*MERCADOL</t>
         </is>
       </c>
-      <c r="E17" s="7" t="n">
+      <c r="E18" s="23" t="n">
         <v>233.62</v>
       </c>
-      <c r="F17" s="6" t="inlineStr">
-        <is>
-          <t>A VISTA</t>
-        </is>
-      </c>
-      <c r="G17" s="6" t="n"/>
-      <c r="H17" s="3" t="n"/>
-      <c r="I17" s="6" t="n"/>
-      <c r="J17" s="3" t="n"/>
-      <c r="K17" s="3" t="n"/>
-    </row>
-    <row r="18" ht="18" customHeight="1">
-      <c r="A18" s="5" t="n"/>
-      <c r="B18" s="6" t="n"/>
-      <c r="C18" s="3" t="n"/>
-      <c r="D18" s="3" t="n"/>
-      <c r="E18" s="7" t="n"/>
-      <c r="F18" s="6" t="inlineStr">
-        <is>
-          <t>A VISTA</t>
-        </is>
-      </c>
-      <c r="G18" s="6" t="n"/>
-      <c r="H18" s="3" t="n"/>
-      <c r="I18" s="6" t="n"/>
-      <c r="J18" s="3" t="n"/>
-      <c r="K18" s="3" t="n"/>
+      <c r="F18" s="21" t="inlineStr">
+        <is>
+          <t>A VISTA</t>
+        </is>
+      </c>
+      <c r="G18" s="21" t="n"/>
+      <c r="H18" s="22" t="n"/>
+      <c r="I18" s="21" t="n"/>
+      <c r="J18" s="22" t="n"/>
+      <c r="K18" s="22" t="n"/>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="5" t="n"/>
@@ -1562,9 +1730,6 @@
           <t>SUB TOTAL</t>
         </is>
       </c>
-      <c r="B55" s="18" t="n"/>
-      <c r="C55" s="18" t="n"/>
-      <c r="D55" s="19" t="n"/>
       <c r="E55" s="10">
         <f>SUM(E5:E54)</f>
         <v/>
@@ -1582,16 +1747,6 @@
           <t>INTERNATIONAL PURCHASES</t>
         </is>
       </c>
-      <c r="B56" s="18" t="n"/>
-      <c r="C56" s="18" t="n"/>
-      <c r="D56" s="18" t="n"/>
-      <c r="E56" s="18" t="n"/>
-      <c r="F56" s="18" t="n"/>
-      <c r="G56" s="18" t="n"/>
-      <c r="H56" s="18" t="n"/>
-      <c r="I56" s="18" t="n"/>
-      <c r="J56" s="18" t="n"/>
-      <c r="K56" s="19" t="n"/>
     </row>
     <row r="57" ht="18" customHeight="1">
       <c r="A57" s="5" t="n"/>
@@ -1684,9 +1839,6 @@
           <t>SUB TOTAL</t>
         </is>
       </c>
-      <c r="B62" s="18" t="n"/>
-      <c r="C62" s="18" t="n"/>
-      <c r="D62" s="19" t="n"/>
       <c r="E62" s="10">
         <f>SUM(E57:E61)</f>
         <v/>
@@ -1704,9 +1856,6 @@
           <t>Annuity installment:</t>
         </is>
       </c>
-      <c r="B63" s="18" t="n"/>
-      <c r="C63" s="18" t="n"/>
-      <c r="D63" s="19" t="n"/>
       <c r="E63" s="7" t="n">
         <v>18.75</v>
       </c>
@@ -1723,9 +1872,6 @@
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B64" s="18" t="n"/>
-      <c r="C64" s="18" t="n"/>
-      <c r="D64" s="19" t="n"/>
       <c r="E64" s="16">
         <f>E55+E62+E63</f>
         <v/>
@@ -1745,18 +1891,12 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="11">
+  <mergeCells count="5">
     <mergeCell ref="C2:K2"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A62:D62"/>
-    <mergeCell ref="A55:D55"/>
-    <mergeCell ref="A64:D64"/>
     <mergeCell ref="C3:K3"/>
-    <mergeCell ref="A63:D63"/>
-    <mergeCell ref="A66:K66"/>
     <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A56:K56"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>